<commit_message>
Add gram-positive bacteria eval
</commit_message>
<xml_diff>
--- a/statistics_general_number_of_bacteria.xlsx
+++ b/statistics_general_number_of_bacteria.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vasav\OneDrive\Рабочий стол\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dmyboi\PycharmProjects\microbiology_diploma\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E879C77-F5B3-4FED-8A54-731D5BB1C208}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{750EC3DA-5C2C-466A-B234-069B8941DE26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1125" yWindow="1125" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -331,9 +331,6 @@
     <t>CLED</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>Cetr</t>
   </si>
   <si>
@@ -953,7 +950,7 @@
         <family val="1"/>
         <charset val="238"/>
       </rPr>
-      <t>sp. LB1-10</t>
+      <t>sp. strain LaBFS2205</t>
     </r>
   </si>
   <si>
@@ -968,97 +965,120 @@
         <family val="1"/>
         <charset val="238"/>
       </rPr>
-      <t>sp. strain LaBFS2205</t>
-    </r>
-  </si>
-  <si>
-    <r>
+      <t>sp. strain CA15-34</t>
+    </r>
+  </si>
+  <si>
+    <t>Przezroczysty, różowy</t>
+  </si>
+  <si>
+    <t>Moellerella wisconsensis</t>
+  </si>
+  <si>
+    <t>Uncultured bacterium AKT-M3_11</t>
+  </si>
+  <si>
+    <t>Uncultured bacterium clone TSCW_OTU_213</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Leclercia </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="238"/>
+      </rPr>
+      <t>sp. G3L</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Citrobacter </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="238"/>
+      </rPr>
+      <t>sp. strain BIGb0161</t>
+    </r>
+  </si>
+  <si>
+    <t>Uncultured bacterium clone Espejo</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Buttiauxella </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="238"/>
+      </rPr>
+      <t>sp. strain HR94</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Kluyvera </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="238"/>
+      </rPr>
+      <t>intermedia strain 0PLS1.17</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="238"/>
+      </rPr>
       <t xml:space="preserve">Erwinia </t>
     </r>
     <r>
       <rPr>
         <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="238"/>
-      </rPr>
-      <t>sp. strain CA15-34</t>
-    </r>
-  </si>
-  <si>
-    <t>Przezroczysty, różowy</t>
-  </si>
-  <si>
-    <t>Moellerella wisconsensis</t>
-  </si>
-  <si>
-    <t>Uncultured bacterium AKT-M3_11</t>
-  </si>
-  <si>
-    <t>Uncultured bacterium clone TSCW_OTU_213</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Leclercia </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="238"/>
-      </rPr>
-      <t>sp. G3L</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Citrobacter </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="238"/>
-      </rPr>
-      <t>sp. strain BIGb0161</t>
-    </r>
-  </si>
-  <si>
-    <t>Uncultured bacterium clone Espejo</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Buttiauxella </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="238"/>
-      </rPr>
-      <t>sp. strain HR94</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Kluyvera </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="238"/>
-      </rPr>
-      <t>intermedia strain 0PLS1.17</t>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="238"/>
+      </rPr>
+      <t>sp. W01</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Pantoea agglomerans </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">strain ASB1 </t>
     </r>
   </si>
 </sst>
@@ -1066,7 +1086,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1126,6 +1146,21 @@
       <family val="1"/>
       <charset val="238"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="238"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -1141,7 +1176,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -1336,11 +1371,29 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1417,43 +1470,50 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1737,9 +1797,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F34"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1759,7 +1819,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -1779,7 +1839,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6">
         <v>2</v>
       </c>
@@ -1799,7 +1859,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -1819,7 +1879,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="6">
         <v>4</v>
       </c>
@@ -1839,7 +1899,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -1859,7 +1919,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="6">
         <v>6</v>
       </c>
@@ -1879,7 +1939,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>7</v>
       </c>
@@ -1899,7 +1959,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="6">
         <v>8</v>
       </c>
@@ -1919,7 +1979,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>9</v>
       </c>
@@ -1939,7 +1999,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="6">
         <v>10</v>
       </c>
@@ -1959,7 +2019,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
         <v>11</v>
       </c>
@@ -1979,7 +2039,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="6">
         <v>12</v>
       </c>
@@ -1999,7 +2059,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
         <v>13</v>
       </c>
@@ -2019,7 +2079,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="6">
         <v>14</v>
       </c>
@@ -2037,7 +2097,7 @@
       </c>
       <c r="F15" s="8"/>
     </row>
-    <row r="16" spans="1:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4">
         <v>15</v>
       </c>
@@ -2055,7 +2115,7 @@
       </c>
       <c r="F16" s="9"/>
     </row>
-    <row r="17" spans="1:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="6">
         <v>16</v>
       </c>
@@ -2073,7 +2133,7 @@
       </c>
       <c r="F17" s="8"/>
     </row>
-    <row r="18" spans="1:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4">
         <v>17</v>
       </c>
@@ -2091,7 +2151,7 @@
       </c>
       <c r="F18" s="9"/>
     </row>
-    <row r="19" spans="1:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="6">
         <v>18</v>
       </c>
@@ -2109,7 +2169,7 @@
       </c>
       <c r="F19" s="8"/>
     </row>
-    <row r="20" spans="1:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4">
         <v>19</v>
       </c>
@@ -2127,7 +2187,7 @@
       </c>
       <c r="F20" s="9"/>
     </row>
-    <row r="21" spans="1:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6">
         <v>20</v>
       </c>
@@ -2145,7 +2205,7 @@
       </c>
       <c r="F21" s="8"/>
     </row>
-    <row r="22" spans="1:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4">
         <v>21</v>
       </c>
@@ -2163,7 +2223,7 @@
       </c>
       <c r="F22" s="9"/>
     </row>
-    <row r="23" spans="1:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="6">
         <v>22</v>
       </c>
@@ -2181,7 +2241,7 @@
       </c>
       <c r="F23" s="8"/>
     </row>
-    <row r="24" spans="1:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="4">
         <v>23</v>
       </c>
@@ -2199,7 +2259,7 @@
       </c>
       <c r="F24" s="9"/>
     </row>
-    <row r="25" spans="1:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="6">
         <v>24</v>
       </c>
@@ -2217,7 +2277,7 @@
       </c>
       <c r="F25" s="8"/>
     </row>
-    <row r="26" spans="1:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4">
         <v>25</v>
       </c>
@@ -2235,7 +2295,7 @@
       </c>
       <c r="F26" s="9"/>
     </row>
-    <row r="27" spans="1:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="6">
         <v>26</v>
       </c>
@@ -2253,7 +2313,7 @@
       </c>
       <c r="F27" s="8"/>
     </row>
-    <row r="28" spans="1:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4">
         <v>27</v>
       </c>
@@ -2271,7 +2331,7 @@
       </c>
       <c r="F28" s="9"/>
     </row>
-    <row r="29" spans="1:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="6">
         <v>28</v>
       </c>
@@ -2289,7 +2349,7 @@
       </c>
       <c r="F29" s="8"/>
     </row>
-    <row r="30" spans="1:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4">
         <v>29</v>
       </c>
@@ -2307,7 +2367,7 @@
       </c>
       <c r="F30" s="9"/>
     </row>
-    <row r="31" spans="1:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="6">
         <v>30</v>
       </c>
@@ -2325,7 +2385,7 @@
       </c>
       <c r="F31" s="8"/>
     </row>
-    <row r="32" spans="1:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4">
         <v>31</v>
       </c>
@@ -2343,7 +2403,7 @@
       </c>
       <c r="F32" s="9"/>
     </row>
-    <row r="33" spans="1:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="6">
         <v>32</v>
       </c>
@@ -2361,7 +2421,7 @@
       </c>
       <c r="F33" s="8"/>
     </row>
-    <row r="34" spans="1:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4">
         <v>33</v>
       </c>
@@ -2386,10 +2446,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69EF5413-6C05-4AD5-AB0D-86080543EAA9}">
-  <dimension ref="A1:C81"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C83"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="31.42578125" customWidth="1"/>
+    <col min="2" max="2" width="25.140625" customWidth="1"/>
+    <col min="3" max="3" width="27.42578125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
         <v>96</v>
       </c>
@@ -2400,852 +2465,863 @@
         <v>98</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="27" t="s">
+    <row r="2" spans="1:3" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="30" t="s">
         <v>99</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="12"/>
+      <c r="C2" s="13"/>
+    </row>
+    <row r="3" spans="1:3" ht="48" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="36"/>
+      <c r="B3" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="48" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="36"/>
+      <c r="B4" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="126.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="29"/>
+      <c r="B5" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="48" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="48" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="48" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="48" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="63.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="63.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="63.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="63.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="48" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="28" t="s">
+        <v>123</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="29"/>
+      <c r="B16" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="79.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="36"/>
+      <c r="B19" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="63.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="29"/>
+      <c r="B20" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="B22" s="40" t="s">
+        <v>105</v>
+      </c>
+      <c r="C22" s="41" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="C23" s="17" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="B28" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="C28" s="17" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="B29" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="C29" s="20" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="33" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="B30" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="C30" s="17" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="26" t="s">
+        <v>141</v>
+      </c>
+      <c r="B31" s="21" t="s">
         <v>100</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C31" s="22" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="48" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="37"/>
+      <c r="B32" s="21" t="s">
+        <v>105</v>
+      </c>
+      <c r="C32" s="22" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="37"/>
+      <c r="B33" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="C33" s="22" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="27"/>
+      <c r="B34" s="21" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="26"/>
-      <c r="B3" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="C3" s="13" t="s">
+      <c r="C34" s="22" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="23" t="s">
+        <v>145</v>
+      </c>
+      <c r="B35" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="C35" s="22" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="23" t="s">
+        <v>146</v>
+      </c>
+      <c r="B36" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="C36" s="22" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="23" t="s">
+        <v>147</v>
+      </c>
+      <c r="B37" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="C37" s="22" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="B38" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="C38" s="22" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="23" t="s">
+        <v>149</v>
+      </c>
+      <c r="B39" s="21" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="26"/>
-      <c r="B4" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="C4" s="13" t="s">
+      <c r="C39" s="22" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="23" t="s">
+        <v>151</v>
+      </c>
+      <c r="B40" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="C40" s="22" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="23" t="s">
+        <v>152</v>
+      </c>
+      <c r="B41" s="21" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="125.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="28"/>
-      <c r="B5" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="63" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="14" t="s">
+      <c r="C41" s="22" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="23" t="s">
+        <v>154</v>
+      </c>
+      <c r="B42" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="C42" s="22" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="38" t="s">
+        <v>155</v>
+      </c>
+      <c r="B43" s="21" t="s">
+        <v>100</v>
+      </c>
+      <c r="C43" s="22" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="37"/>
+      <c r="B44" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="C44" s="22" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="27"/>
+      <c r="B45" s="21" t="s">
+        <v>105</v>
+      </c>
+      <c r="C45" s="22" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="38" t="s">
+        <v>156</v>
+      </c>
+      <c r="B46" s="21" t="s">
+        <v>100</v>
+      </c>
+      <c r="C46" s="22" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="37"/>
+      <c r="B47" s="21" t="s">
+        <v>105</v>
+      </c>
+      <c r="C47" s="22" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="27"/>
+      <c r="B48" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="C48" s="22" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="23" t="s">
+        <v>157</v>
+      </c>
+      <c r="B49" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="C49" s="22" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="23" t="s">
+        <v>158</v>
+      </c>
+      <c r="B50" s="21" t="s">
+        <v>100</v>
+      </c>
+      <c r="C50" s="22" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="23" t="s">
+        <v>154</v>
+      </c>
+      <c r="B51" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="C51" s="22" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="23" t="s">
+        <v>159</v>
+      </c>
+      <c r="B52" s="21" t="s">
+        <v>105</v>
+      </c>
+      <c r="C52" s="22" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="18" t="s">
+        <v>160</v>
+      </c>
+      <c r="B53" s="19" t="s">
+        <v>105</v>
+      </c>
+      <c r="C53" s="20" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" ht="48.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="24" t="s">
+        <v>161</v>
+      </c>
+      <c r="B54" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="C54" s="17" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" ht="33" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="18" t="s">
+        <v>162</v>
+      </c>
+      <c r="B55" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="C55" s="20" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" ht="30.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="B56" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="C56" s="17" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="26" t="s">
+        <v>164</v>
+      </c>
+      <c r="B57" s="21" t="s">
+        <v>105</v>
+      </c>
+      <c r="C57" s="22" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="27"/>
+      <c r="B58" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="C58" s="20" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="28" t="s">
+        <v>165</v>
+      </c>
+      <c r="B59" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="C59" s="13" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="29"/>
+      <c r="B60" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="C60" s="17" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="23" t="s">
+        <v>167</v>
+      </c>
+      <c r="B61" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="C61" s="22" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="B62" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="C62" s="20" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="15" t="s">
+        <v>169</v>
+      </c>
+      <c r="B63" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="C63" s="17" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="23" t="s">
+        <v>171</v>
+      </c>
+      <c r="B64" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="C64" s="22" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="18" t="s">
+        <v>172</v>
+      </c>
+      <c r="B65" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="C65" s="20" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="B66" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="C66" s="17" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="23" t="s">
+        <v>174</v>
+      </c>
+      <c r="B67" s="21" t="s">
+        <v>105</v>
+      </c>
+      <c r="C67" s="22" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="39" t="s">
+        <v>187</v>
+      </c>
+      <c r="B68" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="C68" s="22" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="23" t="s">
+        <v>176</v>
+      </c>
+      <c r="B69" s="21" t="s">
+        <v>105</v>
+      </c>
+      <c r="C69" s="22" t="s">
         <v>108</v>
       </c>
-      <c r="B6" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C6" s="13" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="63" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="14" t="s">
+    </row>
+    <row r="70" spans="1:3" ht="46.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="18" t="s">
+        <v>177</v>
+      </c>
+      <c r="B70" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="C70" s="20" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="30" t="s">
+        <v>179</v>
+      </c>
+      <c r="B71" s="12"/>
+      <c r="C71" s="13"/>
+    </row>
+    <row r="72" spans="1:3" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="29"/>
+      <c r="B72" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="C72" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="B7" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="63" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="14" t="s">
-        <v>112</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="63" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="14" t="s">
-        <v>114</v>
-      </c>
-      <c r="B9" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="78.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="B10" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="78.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="14" t="s">
-        <v>117</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="78.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="14" t="s">
-        <v>118</v>
-      </c>
-      <c r="B12" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="C12" s="13" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="63" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="B14" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="29" t="s">
+    </row>
+    <row r="73" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="31" t="s">
+        <v>180</v>
+      </c>
+      <c r="B73" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="C73" s="22" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="32"/>
+      <c r="B74" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="C74" s="22" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" ht="77.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A75" s="33"/>
+      <c r="B75" s="19"/>
+      <c r="C75" s="20"/>
+    </row>
+    <row r="76" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="34" t="s">
+        <v>181</v>
+      </c>
+      <c r="B76" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="C76" s="13" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A77" s="35"/>
+      <c r="B77" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="C77" s="17" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A78" s="18" t="s">
+        <v>182</v>
+      </c>
+      <c r="B78" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="C78" s="20" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="B79" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="C79" s="17" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" ht="33" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="25" t="s">
+        <v>184</v>
+      </c>
+      <c r="B80" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="C80" s="20" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="B81" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="C81" s="17" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" ht="33" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A82" s="18" t="s">
+        <v>186</v>
+      </c>
+      <c r="B82" s="19" t="s">
+        <v>105</v>
+      </c>
+      <c r="C82" s="20" t="s">
         <v>124</v>
       </c>
-      <c r="B15" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="28"/>
-      <c r="B16" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="78.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="B17" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="29" t="s">
-        <v>129</v>
-      </c>
-      <c r="B18" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="C18" s="13" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="26"/>
-      <c r="B19" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="C19" s="13" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="63" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="28"/>
-      <c r="B20" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C20" s="13" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="78.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="B21" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C21" s="13" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="78.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="B22" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="C22" s="13" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="63" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="14" t="s">
-        <v>133</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="C23" s="13" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="63" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="B24" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="C24" s="13" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="63" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="C25" s="13" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="15" t="s">
-        <v>138</v>
-      </c>
-      <c r="B26" s="16" t="s">
-        <v>104</v>
-      </c>
-      <c r="C26" s="17" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" ht="63.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="B27" s="19" t="s">
-        <v>104</v>
-      </c>
-      <c r="C27" s="20" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" ht="94.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="15" t="s">
-        <v>141</v>
-      </c>
-      <c r="B28" s="16" t="s">
-        <v>102</v>
-      </c>
-      <c r="C28" s="17" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" ht="32.4" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="31" t="s">
-        <v>142</v>
-      </c>
-      <c r="B29" s="21" t="s">
-        <v>100</v>
-      </c>
-      <c r="C29" s="22" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" ht="125.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="30"/>
-      <c r="B30" s="21" t="s">
-        <v>106</v>
-      </c>
-      <c r="C30" s="22" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="30"/>
-      <c r="B31" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="C31" s="22" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="32"/>
-      <c r="B32" s="21" t="s">
-        <v>102</v>
-      </c>
-      <c r="C32" s="22" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="63" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="23" t="s">
-        <v>146</v>
-      </c>
-      <c r="B33" s="21" t="s">
-        <v>102</v>
-      </c>
-      <c r="C33" s="22" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" ht="63" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="23" t="s">
-        <v>147</v>
-      </c>
-      <c r="B34" s="21" t="s">
-        <v>102</v>
-      </c>
-      <c r="C34" s="22" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" ht="63" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="23" t="s">
-        <v>148</v>
-      </c>
-      <c r="B35" s="21" t="s">
-        <v>102</v>
-      </c>
-      <c r="C35" s="22" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="63" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="23" t="s">
-        <v>149</v>
-      </c>
-      <c r="B36" s="21" t="s">
-        <v>102</v>
-      </c>
-      <c r="C36" s="22" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="23" t="s">
-        <v>150</v>
-      </c>
-      <c r="B37" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="C37" s="22" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" ht="63" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="23" t="s">
-        <v>152</v>
-      </c>
-      <c r="B38" s="21" t="s">
-        <v>102</v>
-      </c>
-      <c r="C38" s="22" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" ht="94.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="23" t="s">
-        <v>153</v>
-      </c>
-      <c r="B39" s="21" t="s">
-        <v>106</v>
-      </c>
-      <c r="C39" s="22" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="78.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="23" t="s">
-        <v>155</v>
-      </c>
-      <c r="B40" s="21" t="s">
-        <v>102</v>
-      </c>
-      <c r="C40" s="22" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="33" t="s">
-        <v>156</v>
-      </c>
-      <c r="B41" s="21" t="s">
-        <v>100</v>
-      </c>
-      <c r="C41" s="22" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="30"/>
-      <c r="B42" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="C42" s="22" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="32"/>
-      <c r="B43" s="21" t="s">
-        <v>106</v>
-      </c>
-      <c r="C43" s="22" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="33" t="s">
-        <v>157</v>
-      </c>
-      <c r="B44" s="21" t="s">
-        <v>100</v>
-      </c>
-      <c r="C44" s="22" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="30"/>
-      <c r="B45" s="21" t="s">
-        <v>106</v>
-      </c>
-      <c r="C45" s="22" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="32"/>
-      <c r="B46" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="C46" s="22" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" ht="78.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="23" t="s">
-        <v>158</v>
-      </c>
-      <c r="B47" s="21" t="s">
-        <v>102</v>
-      </c>
-      <c r="C47" s="22" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" ht="63" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="23" t="s">
-        <v>159</v>
-      </c>
-      <c r="B48" s="21" t="s">
-        <v>100</v>
-      </c>
-      <c r="C48" s="22" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" ht="78.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="23" t="s">
-        <v>155</v>
-      </c>
-      <c r="B49" s="21" t="s">
-        <v>102</v>
-      </c>
-      <c r="C49" s="22" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" ht="94.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="23" t="s">
-        <v>160</v>
-      </c>
-      <c r="B50" s="21" t="s">
-        <v>106</v>
-      </c>
-      <c r="C50" s="22" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" ht="78.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="18" t="s">
-        <v>161</v>
-      </c>
-      <c r="B51" s="19" t="s">
-        <v>106</v>
-      </c>
-      <c r="C51" s="20" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" ht="157.19999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="24" t="s">
-        <v>162</v>
-      </c>
-      <c r="B52" s="16" t="s">
-        <v>102</v>
-      </c>
-      <c r="C52" s="17" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" ht="110.4" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="18" t="s">
-        <v>163</v>
-      </c>
-      <c r="B53" s="19" t="s">
-        <v>104</v>
-      </c>
-      <c r="C53" s="20" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" ht="63.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="15" t="s">
-        <v>164</v>
-      </c>
-      <c r="B54" s="16" t="s">
-        <v>100</v>
-      </c>
-      <c r="C54" s="17" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" ht="30.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="31" t="s">
-        <v>165</v>
-      </c>
-      <c r="B55" s="21" t="s">
-        <v>106</v>
-      </c>
-      <c r="C55" s="22" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="32"/>
-      <c r="B56" s="19" t="s">
-        <v>104</v>
-      </c>
-      <c r="C56" s="20" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" ht="30.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A57" s="29" t="s">
-        <v>166</v>
-      </c>
-      <c r="B57" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="C57" s="13" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A58" s="28"/>
-      <c r="B58" s="16" t="s">
-        <v>106</v>
-      </c>
-      <c r="C58" s="17" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A59" s="23" t="s">
-        <v>168</v>
-      </c>
-      <c r="B59" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="C59" s="22" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" ht="63" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A60" s="18" t="s">
-        <v>169</v>
-      </c>
-      <c r="B60" s="19" t="s">
-        <v>102</v>
-      </c>
-      <c r="C60" s="20" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" ht="79.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A61" s="15" t="s">
-        <v>170</v>
-      </c>
-      <c r="B61" s="16" t="s">
-        <v>104</v>
-      </c>
-      <c r="C61" s="17" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" ht="48" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A62" s="23" t="s">
-        <v>172</v>
-      </c>
-      <c r="B62" s="21" t="s">
-        <v>102</v>
-      </c>
-      <c r="C62" s="22" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" ht="94.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A63" s="18" t="s">
-        <v>173</v>
-      </c>
-      <c r="B63" s="19" t="s">
-        <v>102</v>
-      </c>
-      <c r="C63" s="20" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" ht="48" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A64" s="15" t="s">
-        <v>174</v>
-      </c>
-      <c r="B64" s="16" t="s">
-        <v>106</v>
-      </c>
-      <c r="C64" s="17" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" ht="32.4" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A65" s="23" t="s">
-        <v>175</v>
-      </c>
-      <c r="B65" s="21" t="s">
-        <v>106</v>
-      </c>
-      <c r="C65" s="22" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A66" s="23" t="s">
-        <v>177</v>
-      </c>
-      <c r="B66" s="21" t="s">
-        <v>102</v>
-      </c>
-      <c r="C66" s="22" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" ht="78.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A67" s="23" t="s">
-        <v>178</v>
-      </c>
-      <c r="B67" s="21" t="s">
-        <v>106</v>
-      </c>
-      <c r="C67" s="22" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" ht="78.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A68" s="18" t="s">
-        <v>179</v>
-      </c>
-      <c r="B68" s="19" t="s">
-        <v>104</v>
-      </c>
-      <c r="C68" s="20" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" ht="46.2" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A69" s="27" t="s">
-        <v>181</v>
-      </c>
-      <c r="B69" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="C69" s="13" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A70" s="28"/>
-      <c r="B70" s="16" t="s">
-        <v>104</v>
-      </c>
-      <c r="C70" s="17" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A71" s="35" t="s">
-        <v>182</v>
-      </c>
-      <c r="B71" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="C71" s="22" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A72" s="34"/>
-      <c r="B72" s="21" t="s">
-        <v>102</v>
-      </c>
-      <c r="C72" s="22" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A73" s="36"/>
-      <c r="B73" s="19" t="s">
-        <v>106</v>
-      </c>
-      <c r="C73" s="20" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" ht="77.400000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A74" s="37" t="s">
-        <v>183</v>
-      </c>
-      <c r="B74" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C74" s="13" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A75" s="38"/>
-      <c r="B75" s="16" t="s">
-        <v>102</v>
-      </c>
-      <c r="C75" s="17" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A76" s="18" t="s">
-        <v>184</v>
-      </c>
-      <c r="B76" s="19" t="s">
-        <v>104</v>
-      </c>
-      <c r="C76" s="20" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" ht="79.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A77" s="15" t="s">
-        <v>185</v>
-      </c>
-      <c r="B77" s="16" t="s">
-        <v>106</v>
-      </c>
-      <c r="C77" s="17" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" ht="79.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A78" s="25" t="s">
-        <v>186</v>
-      </c>
-      <c r="B78" s="19" t="s">
-        <v>104</v>
-      </c>
-      <c r="C78" s="20" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" ht="63.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A79" s="15" t="s">
-        <v>187</v>
-      </c>
-      <c r="B79" s="16" t="s">
-        <v>104</v>
-      </c>
-      <c r="C79" s="17" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" ht="94.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A80" s="18" t="s">
-        <v>188</v>
-      </c>
-      <c r="B80" s="19" t="s">
-        <v>106</v>
-      </c>
-      <c r="C80" s="20" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="81" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    </row>
+    <row r="83" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A55:A56"/>
-    <mergeCell ref="A57:A58"/>
-    <mergeCell ref="A69:A70"/>
-    <mergeCell ref="A71:A73"/>
-    <mergeCell ref="A74:A75"/>
+    <mergeCell ref="A46:A48"/>
     <mergeCell ref="A2:A5"/>
     <mergeCell ref="A15:A16"/>
     <mergeCell ref="A18:A20"/>
-    <mergeCell ref="A29:A32"/>
-    <mergeCell ref="A41:A43"/>
-    <mergeCell ref="A44:A46"/>
+    <mergeCell ref="A31:A34"/>
+    <mergeCell ref="A43:A45"/>
+    <mergeCell ref="A57:A58"/>
+    <mergeCell ref="A59:A60"/>
+    <mergeCell ref="A71:A72"/>
+    <mergeCell ref="A73:A75"/>
+    <mergeCell ref="A76:A77"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>